<commit_message>
Crosschecked and verfied All Things
</commit_message>
<xml_diff>
--- a/sbom_output/public/sbom_report.xlsx
+++ b/sbom_output/public/sbom_report.xlsx
@@ -71,13 +71,13 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00000000"/>
       <sz val="9"/>
     </font>
     <font>
@@ -156,8 +156,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC107"/>
-        <bgColor rgb="00FFC107"/>
+        <fgColor rgb="004CAF50"/>
+        <bgColor rgb="004CAF50"/>
       </patternFill>
     </fill>
     <fill>
@@ -170,6 +170,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FF4C4C"/>
         <bgColor rgb="00FF4C4C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC107"/>
+        <bgColor rgb="00FFC107"/>
       </patternFill>
     </fill>
     <fill>
@@ -194,12 +200,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFCDD2"/>
         <bgColor rgb="00FFCDD2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004CAF50"/>
-        <bgColor rgb="004CAF50"/>
       </patternFill>
     </fill>
   </fills>
@@ -229,7 +229,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -296,10 +296,13 @@
     <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -309,13 +312,13 @@
     <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -325,13 +328,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -723,7 +726,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CycloneDX v1.7 | Generated: 2026-06-26T06:14:55Z | Report Date: 2026-06-26 11:44</t>
+          <t>CycloneDX v1.7 | Generated: 2026-06-26T09:25:48Z | Report Date: 2026-06-26 14:55</t>
         </is>
       </c>
     </row>
@@ -756,12 +759,12 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -868,7 +871,7 @@
       </c>
       <c r="E9" s="21" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F9" s="20" t="inlineStr">
@@ -938,7 +941,7 @@
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="F11" s="20" t="inlineStr">
@@ -971,7 +974,7 @@
           <t>Apache-2.0</t>
         </is>
       </c>
-      <c r="E12" s="21" t="inlineStr">
+      <c r="E12" s="25" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -1006,7 +1009,7 @@
           <t>Apache-2.0</t>
         </is>
       </c>
-      <c r="E13" s="25" t="inlineStr">
+      <c r="E13" s="26" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1041,7 +1044,7 @@
           <t>Apache-2.0</t>
         </is>
       </c>
-      <c r="E14" s="25" t="inlineStr">
+      <c r="E14" s="26" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -1073,7 +1076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:AC10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1090,27 +1093,34 @@
     <col width="25" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="45" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="45" customWidth="1" min="16" max="16"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
     <col width="45" customWidth="1" min="17" max="17"/>
-    <col width="23" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="19" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="34" customWidth="1" min="22" max="22"/>
+    <col width="45" customWidth="1" min="18" max="18"/>
+    <col width="23" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="37" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="34" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="45" customWidth="1" min="26" max="26"/>
+    <col width="22" customWidth="1" min="27" max="27"/>
+    <col width="45" customWidth="1" min="28" max="28"/>
+    <col width="23" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
-        <is>
-          <t>SBOM Component Data - All 21 Client Attributes</t>
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>SBOM Component Data - All 21 Client Attributes + Enterprise Enhancements</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Author: Compliance &amp; Enrichment Specialist (Team Member 3)  |  Generated: 2026-06-26T06:14:55Z</t>
+          <t>Author: Compliance &amp; Enrichment Specialist (Team Member 3)  |  Generated: 2026-06-26T09:25:48Z</t>
         </is>
       </c>
     </row>
@@ -1183,47 +1193,82 @@
       </c>
       <c r="N4" s="18" t="inlineStr">
         <is>
+          <t>Criticality Reason</t>
+        </is>
+      </c>
+      <c r="O4" s="18" t="inlineStr">
+        <is>
           <t>Usage Restrictions</t>
         </is>
       </c>
-      <c r="O4" s="18" t="inlineStr">
+      <c r="P4" s="18" t="inlineStr">
         <is>
           <t>Checksums or Hashes</t>
         </is>
       </c>
-      <c r="P4" s="18" t="inlineStr">
+      <c r="Q4" s="18" t="inlineStr">
         <is>
           <t>Comments or Notes</t>
         </is>
       </c>
-      <c r="Q4" s="18" t="inlineStr">
+      <c r="R4" s="18" t="inlineStr">
         <is>
           <t>Author of SBOM Data</t>
         </is>
       </c>
-      <c r="R4" s="18" t="inlineStr">
+      <c r="S4" s="18" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="S4" s="18" t="inlineStr">
+      <c r="T4" s="18" t="inlineStr">
         <is>
           <t>Executable Property</t>
         </is>
       </c>
-      <c r="T4" s="18" t="inlineStr">
+      <c r="U4" s="18" t="inlineStr">
+        <is>
+          <t>Executable Evidence</t>
+        </is>
+      </c>
+      <c r="V4" s="18" t="inlineStr">
         <is>
           <t>Archive Property</t>
         </is>
       </c>
-      <c r="U4" s="18" t="inlineStr">
+      <c r="W4" s="18" t="inlineStr">
         <is>
           <t>Structured Property</t>
         </is>
       </c>
-      <c r="V4" s="18" t="inlineStr">
+      <c r="X4" s="18" t="inlineStr">
         <is>
           <t>Unique Identifier (PURL)</t>
+        </is>
+      </c>
+      <c r="Y4" s="18" t="inlineStr">
+        <is>
+          <t>Trust Score</t>
+        </is>
+      </c>
+      <c r="Z4" s="18" t="inlineStr">
+        <is>
+          <t>Trust Score Reasons</t>
+        </is>
+      </c>
+      <c r="AA4" s="18" t="inlineStr">
+        <is>
+          <t>Repository Registry</t>
+        </is>
+      </c>
+      <c r="AB4" s="18" t="inlineStr">
+        <is>
+          <t>Repository URL</t>
+        </is>
+      </c>
+      <c r="AC4" s="18" t="inlineStr">
+        <is>
+          <t>Repository Ecosystem</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1276,7 @@
       <c r="A5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="28" t="inlineStr">
         <is>
           <t>requirements.txt</t>
         </is>
@@ -1278,62 +1323,99 @@
       </c>
       <c r="K5" s="19" t="inlineStr">
         <is>
-          <t>2026-06-26T06:14:56.141587Z</t>
+          <t>2026-06-26T09:25:49.183802Z</t>
         </is>
       </c>
       <c r="L5" s="19" t="inlineStr">
         <is>
-          <t>2029-06-25T06:14:56Z</t>
+          <t>2029-06-25T09:25:49Z</t>
         </is>
       </c>
       <c r="M5" s="21" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N5" s="20" t="inlineStr">
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="N5" s="19" t="inlineStr">
+        <is>
+          <t>Score 15: component type='application' (+15)</t>
+        </is>
+      </c>
+      <c r="O5" s="20" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="O5" s="20" t="inlineStr">
+      <c r="P5" s="20" t="inlineStr">
         <is>
           <t>SHA-256:5a1746a9ad87d418...</t>
         </is>
       </c>
-      <c r="P5" s="20" t="inlineStr">
+      <c r="Q5" s="20" t="inlineStr">
         <is>
           <t>Scanned and verified library</t>
         </is>
       </c>
-      <c r="Q5" s="19" t="inlineStr">
+      <c r="R5" s="19" t="inlineStr">
         <is>
           <t>Compliance &amp; Enrichment Specialist (Team Member 3)</t>
         </is>
       </c>
-      <c r="R5" s="19" t="inlineStr">
-        <is>
-          <t>2026-06-26T06:14:55Z</t>
-        </is>
-      </c>
-      <c r="S5" s="19" t="inlineStr">
+      <c r="S5" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-26T09:25:48Z</t>
+        </is>
+      </c>
+      <c r="T5" s="20" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="T5" s="19" t="inlineStr">
+      <c r="U5" s="19" t="inlineStr">
+        <is>
+          <t>CycloneDX type=application</t>
+        </is>
+      </c>
+      <c r="V5" s="19" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="U5" s="20" t="inlineStr">
+      <c r="W5" s="20" t="inlineStr">
         <is>
           <t>CycloneDX JSON v1.6</t>
         </is>
       </c>
-      <c r="V5" s="20" t="inlineStr">
+      <c r="X5" s="19" t="inlineStr">
         <is>
           <t>pkg:pypi/requirements.txt@1.0.0</t>
+        </is>
+      </c>
+      <c r="Y5" s="20" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="Z5" s="20" t="inlineStr">
+        <is>
+          <t>+25: Hash/checksum verified
++20: PURL identifier available
++15: License identified (Apache-2.0)</t>
+        </is>
+      </c>
+      <c r="AA5" s="20" t="inlineStr">
+        <is>
+          <t>PyPI</t>
+        </is>
+      </c>
+      <c r="AB5" s="20" t="inlineStr">
+        <is>
+          <t>https://pypi.org/project/requirements.txt/</t>
+        </is>
+      </c>
+      <c r="AC5" s="20" t="inlineStr">
+        <is>
+          <t>Python</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1423,7 @@
       <c r="A6" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>django</t>
         </is>
@@ -1401,49 +1483,88 @@
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="N6" s="23" t="inlineStr">
+      <c r="N6" s="22" t="inlineStr">
+        <is>
+          <t>Manually overridden in config to 'critical'</t>
+        </is>
+      </c>
+      <c r="O6" s="23" t="inlineStr">
         <is>
           <t>Subject to internal framework deployment guidelines</t>
         </is>
       </c>
-      <c r="O6" s="23" t="inlineStr">
+      <c r="P6" s="23" t="inlineStr">
         <is>
           <t>SHA-256:6a47faad96b2260a...</t>
         </is>
       </c>
-      <c r="P6" s="23" t="inlineStr">
+      <c r="Q6" s="23" t="inlineStr">
         <is>
           <t>Primary web backend framework</t>
         </is>
       </c>
-      <c r="Q6" s="22" t="inlineStr">
+      <c r="R6" s="22" t="inlineStr">
         <is>
           <t>Compliance &amp; Enrichment Specialist (Team Member 3)</t>
         </is>
       </c>
-      <c r="R6" s="22" t="inlineStr">
-        <is>
-          <t>2026-06-26T06:14:55Z</t>
-        </is>
-      </c>
-      <c r="S6" s="22" t="inlineStr">
+      <c r="S6" s="23" t="inlineStr">
+        <is>
+          <t>2026-06-26T09:25:48Z</t>
+        </is>
+      </c>
+      <c r="T6" s="23" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="T6" s="22" t="inlineStr">
+      <c r="U6" s="22" t="inlineStr">
+        <is>
+          <t>PyPI package (typically a library)</t>
+        </is>
+      </c>
+      <c r="V6" s="22" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="U6" s="23" t="inlineStr">
+      <c r="W6" s="23" t="inlineStr">
         <is>
           <t>CycloneDX JSON v1.6</t>
         </is>
       </c>
-      <c r="V6" s="23" t="inlineStr">
+      <c r="X6" s="22" t="inlineStr">
         <is>
           <t>pkg:pypi/django@2.1</t>
+        </is>
+      </c>
+      <c r="Y6" s="23" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Z6" s="23" t="inlineStr">
+        <is>
+          <t>+30: Version confirmed from package registry (API available)
++25: Hash/checksum verified
++20: PURL identifier available
++15: License identified (Apache-2.0)
++10: Manually reviewed in config overrides</t>
+        </is>
+      </c>
+      <c r="AA6" s="23" t="inlineStr">
+        <is>
+          <t>PyPI</t>
+        </is>
+      </c>
+      <c r="AB6" s="23" t="inlineStr">
+        <is>
+          <t>https://pypi.org/project/django/</t>
+        </is>
+      </c>
+      <c r="AC6" s="23" t="inlineStr">
+        <is>
+          <t>Python</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1572,7 @@
       <c r="A7" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="28" t="inlineStr">
         <is>
           <t>jinja2</t>
         </is>
@@ -1508,52 +1629,90 @@
       </c>
       <c r="M7" s="21" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="N7" s="20" t="inlineStr">
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="N7" s="19" t="inlineStr">
+        <is>
+          <t>Score 10: component type='library' (+10)</t>
+        </is>
+      </c>
+      <c r="O7" s="20" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="O7" s="20" t="inlineStr">
+      <c r="P7" s="20" t="inlineStr">
         <is>
           <t>SHA-256:bea121f34d38d518...</t>
         </is>
       </c>
-      <c r="P7" s="20" t="inlineStr">
+      <c r="Q7" s="20" t="inlineStr">
         <is>
           <t>Scanned and verified library</t>
         </is>
       </c>
-      <c r="Q7" s="19" t="inlineStr">
+      <c r="R7" s="19" t="inlineStr">
         <is>
           <t>Compliance &amp; Enrichment Specialist (Team Member 3)</t>
         </is>
       </c>
-      <c r="R7" s="19" t="inlineStr">
-        <is>
-          <t>2026-06-26T06:14:55Z</t>
-        </is>
-      </c>
-      <c r="S7" s="19" t="inlineStr">
+      <c r="S7" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-26T09:25:48Z</t>
+        </is>
+      </c>
+      <c r="T7" s="20" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="T7" s="19" t="inlineStr">
+      <c r="U7" s="19" t="inlineStr">
+        <is>
+          <t>PyPI package (typically a library)</t>
+        </is>
+      </c>
+      <c r="V7" s="19" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="U7" s="20" t="inlineStr">
+      <c r="W7" s="20" t="inlineStr">
         <is>
           <t>CycloneDX JSON v1.6</t>
         </is>
       </c>
-      <c r="V7" s="20" t="inlineStr">
+      <c r="X7" s="19" t="inlineStr">
         <is>
           <t>pkg:pypi/jinja2@2.10</t>
+        </is>
+      </c>
+      <c r="Y7" s="20" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="Z7" s="20" t="inlineStr">
+        <is>
+          <t>+30: Version confirmed from package registry (API available)
++25: Hash/checksum verified
++20: PURL identifier available
++15: License identified (Apache-2.0)</t>
+        </is>
+      </c>
+      <c r="AA7" s="20" t="inlineStr">
+        <is>
+          <t>PyPI</t>
+        </is>
+      </c>
+      <c r="AB7" s="20" t="inlineStr">
+        <is>
+          <t>https://pypi.org/project/jinja2/</t>
+        </is>
+      </c>
+      <c r="AC7" s="20" t="inlineStr">
+        <is>
+          <t>Python</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1720,7 @@
       <c r="A8" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>numpy</t>
         </is>
@@ -1616,54 +1775,93 @@
           <t>2021-07-22T16:03:25Z</t>
         </is>
       </c>
-      <c r="M8" s="21" t="inlineStr">
+      <c r="M8" s="25" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="N8" s="23" t="inlineStr">
+      <c r="N8" s="22" t="inlineStr">
+        <is>
+          <t>Manually overridden in config to 'medium'</t>
+        </is>
+      </c>
+      <c r="O8" s="23" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="O8" s="23" t="inlineStr">
+      <c r="P8" s="23" t="inlineStr">
         <is>
           <t>SHA-256:a890e78aadf77316...</t>
         </is>
       </c>
-      <c r="P8" s="23" t="inlineStr">
+      <c r="Q8" s="23" t="inlineStr">
         <is>
           <t>Numeric and mathematical computation core package</t>
         </is>
       </c>
-      <c r="Q8" s="22" t="inlineStr">
+      <c r="R8" s="22" t="inlineStr">
         <is>
           <t>Compliance &amp; Enrichment Specialist (Team Member 3)</t>
         </is>
       </c>
-      <c r="R8" s="22" t="inlineStr">
-        <is>
-          <t>2026-06-26T06:14:55Z</t>
-        </is>
-      </c>
-      <c r="S8" s="22" t="inlineStr">
+      <c r="S8" s="23" t="inlineStr">
+        <is>
+          <t>2026-06-26T09:25:48Z</t>
+        </is>
+      </c>
+      <c r="T8" s="23" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="T8" s="22" t="inlineStr">
+      <c r="U8" s="22" t="inlineStr">
+        <is>
+          <t>PyPI package (typically a library)</t>
+        </is>
+      </c>
+      <c r="V8" s="22" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="U8" s="23" t="inlineStr">
+      <c r="W8" s="23" t="inlineStr">
         <is>
           <t>CycloneDX JSON v1.6</t>
         </is>
       </c>
-      <c r="V8" s="23" t="inlineStr">
+      <c r="X8" s="22" t="inlineStr">
         <is>
           <t>pkg:pypi/numpy@1.15.0</t>
+        </is>
+      </c>
+      <c r="Y8" s="23" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Z8" s="23" t="inlineStr">
+        <is>
+          <t>+30: Version confirmed from package registry (API available)
++25: Hash/checksum verified
++20: PURL identifier available
++15: License identified (Apache-2.0)
++10: Manually reviewed in config overrides</t>
+        </is>
+      </c>
+      <c r="AA8" s="23" t="inlineStr">
+        <is>
+          <t>PyPI</t>
+        </is>
+      </c>
+      <c r="AB8" s="23" t="inlineStr">
+        <is>
+          <t>https://pypi.org/project/numpy/</t>
+        </is>
+      </c>
+      <c r="AC8" s="23" t="inlineStr">
+        <is>
+          <t>Python</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1869,7 @@
       <c r="A9" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
         <is>
           <t>requests</t>
         </is>
@@ -1726,54 +1924,93 @@
           <t>2021-10-17T15:46:10Z</t>
         </is>
       </c>
-      <c r="M9" s="25" t="inlineStr">
+      <c r="M9" s="26" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="N9" s="20" t="inlineStr">
+      <c r="N9" s="19" t="inlineStr">
+        <is>
+          <t>Manually overridden in config to 'high'</t>
+        </is>
+      </c>
+      <c r="O9" s="20" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="O9" s="20" t="inlineStr">
+      <c r="P9" s="20" t="inlineStr">
         <is>
           <t>SHA-256:29a9bb27fe60f047...</t>
         </is>
       </c>
-      <c r="P9" s="20" t="inlineStr">
+      <c r="Q9" s="20" t="inlineStr">
         <is>
           <t>Critical HTTP client library used for core backend integrations</t>
         </is>
       </c>
-      <c r="Q9" s="19" t="inlineStr">
+      <c r="R9" s="19" t="inlineStr">
         <is>
           <t>Compliance &amp; Enrichment Specialist (Team Member 3)</t>
         </is>
       </c>
-      <c r="R9" s="19" t="inlineStr">
-        <is>
-          <t>2026-06-26T06:14:55Z</t>
-        </is>
-      </c>
-      <c r="S9" s="19" t="inlineStr">
+      <c r="S9" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-26T09:25:48Z</t>
+        </is>
+      </c>
+      <c r="T9" s="20" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="T9" s="19" t="inlineStr">
+      <c r="U9" s="19" t="inlineStr">
+        <is>
+          <t>PyPI package (typically a library)</t>
+        </is>
+      </c>
+      <c r="V9" s="19" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="U9" s="20" t="inlineStr">
+      <c r="W9" s="20" t="inlineStr">
         <is>
           <t>CycloneDX JSON v1.6</t>
         </is>
       </c>
-      <c r="V9" s="20" t="inlineStr">
+      <c r="X9" s="19" t="inlineStr">
         <is>
           <t>pkg:pypi/requests@2.20.0</t>
+        </is>
+      </c>
+      <c r="Y9" s="20" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Z9" s="20" t="inlineStr">
+        <is>
+          <t>+30: Version confirmed from package registry (API available)
++25: Hash/checksum verified
++20: PURL identifier available
++15: License identified (Apache-2.0)
++10: Manually reviewed in config overrides</t>
+        </is>
+      </c>
+      <c r="AA9" s="20" t="inlineStr">
+        <is>
+          <t>PyPI</t>
+        </is>
+      </c>
+      <c r="AB9" s="20" t="inlineStr">
+        <is>
+          <t>https://pypi.org/project/requests/</t>
+        </is>
+      </c>
+      <c r="AC9" s="20" t="inlineStr">
+        <is>
+          <t>Python</t>
         </is>
       </c>
     </row>
@@ -1781,7 +2018,7 @@
       <c r="A10" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>urllib3</t>
         </is>
@@ -1836,61 +2073,100 @@
           <t>2022-04-16T17:49:45Z</t>
         </is>
       </c>
-      <c r="M10" s="25" t="inlineStr">
+      <c r="M10" s="26" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="N10" s="23" t="inlineStr">
+      <c r="N10" s="22" t="inlineStr">
+        <is>
+          <t>Manually overridden in config to 'high'</t>
+        </is>
+      </c>
+      <c r="O10" s="23" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="O10" s="23" t="inlineStr">
+      <c r="P10" s="23" t="inlineStr">
         <is>
           <t>SHA-256:889a9b94b6891674...</t>
         </is>
       </c>
-      <c r="P10" s="23" t="inlineStr">
+      <c r="Q10" s="23" t="inlineStr">
         <is>
           <t>Core networking transport library for HTTP calls</t>
         </is>
       </c>
-      <c r="Q10" s="22" t="inlineStr">
+      <c r="R10" s="22" t="inlineStr">
         <is>
           <t>Compliance &amp; Enrichment Specialist (Team Member 3)</t>
         </is>
       </c>
-      <c r="R10" s="22" t="inlineStr">
-        <is>
-          <t>2026-06-26T06:14:55Z</t>
-        </is>
-      </c>
-      <c r="S10" s="22" t="inlineStr">
+      <c r="S10" s="23" t="inlineStr">
+        <is>
+          <t>2026-06-26T09:25:48Z</t>
+        </is>
+      </c>
+      <c r="T10" s="23" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="T10" s="22" t="inlineStr">
+      <c r="U10" s="22" t="inlineStr">
+        <is>
+          <t>PyPI package (typically a library)</t>
+        </is>
+      </c>
+      <c r="V10" s="22" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="U10" s="23" t="inlineStr">
+      <c r="W10" s="23" t="inlineStr">
         <is>
           <t>CycloneDX JSON v1.6</t>
         </is>
       </c>
-      <c r="V10" s="23" t="inlineStr">
+      <c r="X10" s="22" t="inlineStr">
         <is>
           <t>pkg:pypi/urllib3@1.24.2</t>
+        </is>
+      </c>
+      <c r="Y10" s="23" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="Z10" s="23" t="inlineStr">
+        <is>
+          <t>+30: Version confirmed from package registry (API available)
++25: Hash/checksum verified
++20: PURL identifier available
++15: License identified (Apache-2.0)
++10: Manually reviewed in config overrides</t>
+        </is>
+      </c>
+      <c r="AA10" s="23" t="inlineStr">
+        <is>
+          <t>PyPI</t>
+        </is>
+      </c>
+      <c r="AB10" s="23" t="inlineStr">
+        <is>
+          <t>https://pypi.org/project/urllib3/</t>
+        </is>
+      </c>
+      <c r="AC10" s="23" t="inlineStr">
+        <is>
+          <t>Python</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:V2"/>
-    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A2:AC2"/>
+    <mergeCell ref="A1:AC1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1917,7 +2193,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Vulnerability Matrix</t>
         </is>
@@ -1975,7 +2251,7 @@
           <t>CVE-2018-16984</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2015,7 +2291,7 @@
           <t>CVE-2019-10906</t>
         </is>
       </c>
-      <c r="C5" s="30" t="inlineStr">
+      <c r="C5" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2055,7 +2331,7 @@
           <t>CVE-2019-11236</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2095,7 +2371,7 @@
           <t>CVE-2019-11358</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
+      <c r="C7" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2135,7 +2411,7 @@
           <t>CVE-2019-12308</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2175,7 +2451,7 @@
           <t>CVE-2019-12781</t>
         </is>
       </c>
-      <c r="C9" s="29" t="inlineStr">
+      <c r="C9" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2215,7 +2491,7 @@
           <t>CVE-2019-14232</t>
         </is>
       </c>
-      <c r="C10" s="30" t="inlineStr">
+      <c r="C10" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2255,7 +2531,7 @@
           <t>CVE-2019-14233</t>
         </is>
       </c>
-      <c r="C11" s="30" t="inlineStr">
+      <c r="C11" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2295,7 +2571,7 @@
           <t>CVE-2019-14234</t>
         </is>
       </c>
-      <c r="C12" s="31" t="inlineStr">
+      <c r="C12" s="32" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -2335,7 +2611,7 @@
           <t>CVE-2019-14235</t>
         </is>
       </c>
-      <c r="C13" s="30" t="inlineStr">
+      <c r="C13" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2375,7 +2651,7 @@
           <t>CVE-2019-19118</t>
         </is>
       </c>
-      <c r="C14" s="30" t="inlineStr">
+      <c r="C14" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2415,7 +2691,7 @@
           <t>CVE-2019-19844</t>
         </is>
       </c>
-      <c r="C15" s="31" t="inlineStr">
+      <c r="C15" s="32" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -2455,7 +2731,7 @@
           <t>CVE-2019-3498</t>
         </is>
       </c>
-      <c r="C16" s="30" t="inlineStr">
+      <c r="C16" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2495,7 +2771,7 @@
           <t>CVE-2019-6446</t>
         </is>
       </c>
-      <c r="C17" s="29" t="inlineStr">
+      <c r="C17" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2535,7 +2811,7 @@
           <t>CVE-2019-6975</t>
         </is>
       </c>
-      <c r="C18" s="30" t="inlineStr">
+      <c r="C18" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2575,7 +2851,7 @@
           <t>CVE-2020-26137</t>
         </is>
       </c>
-      <c r="C19" s="29" t="inlineStr">
+      <c r="C19" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2615,7 +2891,7 @@
           <t>CVE-2020-28493</t>
         </is>
       </c>
-      <c r="C20" s="29" t="inlineStr">
+      <c r="C20" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2655,7 +2931,7 @@
           <t>CVE-2020-7471</t>
         </is>
       </c>
-      <c r="C21" s="31" t="inlineStr">
+      <c r="C21" s="32" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -2695,7 +2971,7 @@
           <t>CVE-2021-33203</t>
         </is>
       </c>
-      <c r="C22" s="29" t="inlineStr">
+      <c r="C22" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2735,7 +3011,7 @@
           <t>CVE-2021-33430</t>
         </is>
       </c>
-      <c r="C23" s="29" t="inlineStr">
+      <c r="C23" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2775,7 +3051,7 @@
           <t>CVE-2021-34141</t>
         </is>
       </c>
-      <c r="C24" s="29" t="inlineStr">
+      <c r="C24" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2815,7 +3091,7 @@
           <t>CVE-2021-41495</t>
         </is>
       </c>
-      <c r="C25" s="29" t="inlineStr">
+      <c r="C25" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2855,7 +3131,7 @@
           <t>CVE-2021-41496</t>
         </is>
       </c>
-      <c r="C26" s="29" t="inlineStr">
+      <c r="C26" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2895,7 +3171,7 @@
           <t>CVE-2022-36359</t>
         </is>
       </c>
-      <c r="C27" s="30" t="inlineStr">
+      <c r="C27" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -2935,7 +3211,7 @@
           <t>CVE-2023-32681</t>
         </is>
       </c>
-      <c r="C28" s="29" t="inlineStr">
+      <c r="C28" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -2975,7 +3251,7 @@
           <t>CVE-2023-43804</t>
         </is>
       </c>
-      <c r="C29" s="29" t="inlineStr">
+      <c r="C29" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -3015,7 +3291,7 @@
           <t>CVE-2023-45803</t>
         </is>
       </c>
-      <c r="C30" s="29" t="inlineStr">
+      <c r="C30" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -3055,7 +3331,7 @@
           <t>CVE-2024-22195</t>
         </is>
       </c>
-      <c r="C31" s="29" t="inlineStr">
+      <c r="C31" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -3095,7 +3371,7 @@
           <t>CVE-2024-34064</t>
         </is>
       </c>
-      <c r="C32" s="29" t="inlineStr">
+      <c r="C32" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -3135,7 +3411,7 @@
           <t>CVE-2024-35195</t>
         </is>
       </c>
-      <c r="C33" s="29" t="inlineStr">
+      <c r="C33" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -3175,7 +3451,7 @@
           <t>CVE-2024-37891</t>
         </is>
       </c>
-      <c r="C34" s="29" t="inlineStr">
+      <c r="C34" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -3215,7 +3491,7 @@
           <t>CVE-2024-45231</t>
         </is>
       </c>
-      <c r="C35" s="29" t="inlineStr">
+      <c r="C35" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -3255,7 +3531,7 @@
           <t>CVE-2024-47081</t>
         </is>
       </c>
-      <c r="C36" s="29" t="inlineStr">
+      <c r="C36" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -3295,7 +3571,7 @@
           <t>CVE-2024-56326</t>
         </is>
       </c>
-      <c r="C37" s="30" t="inlineStr">
+      <c r="C37" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -3335,7 +3611,7 @@
           <t>CVE-2025-27516</t>
         </is>
       </c>
-      <c r="C38" s="30" t="inlineStr">
+      <c r="C38" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -3375,7 +3651,7 @@
           <t>CVE-2025-48432</t>
         </is>
       </c>
-      <c r="C39" s="29" t="inlineStr">
+      <c r="C39" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -3415,7 +3691,7 @@
           <t>CVE-2025-50181</t>
         </is>
       </c>
-      <c r="C40" s="29" t="inlineStr">
+      <c r="C40" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -3455,7 +3731,7 @@
           <t>CVE-2025-57833</t>
         </is>
       </c>
-      <c r="C41" s="30" t="inlineStr">
+      <c r="C41" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -3495,7 +3771,7 @@
           <t>CVE-2025-64458</t>
         </is>
       </c>
-      <c r="C42" s="30" t="inlineStr">
+      <c r="C42" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -3536,7 +3812,7 @@
           <t>CVE-2025-64459</t>
         </is>
       </c>
-      <c r="C43" s="31" t="inlineStr">
+      <c r="C43" s="32" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
@@ -3577,7 +3853,7 @@
           <t>CVE-2025-66418</t>
         </is>
       </c>
-      <c r="C44" s="30" t="inlineStr">
+      <c r="C44" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -3617,7 +3893,7 @@
           <t>CVE-2025-66471</t>
         </is>
       </c>
-      <c r="C45" s="30" t="inlineStr">
+      <c r="C45" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -3657,7 +3933,7 @@
           <t>CVE-2026-21441</t>
         </is>
       </c>
-      <c r="C46" s="30" t="inlineStr">
+      <c r="C46" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -3697,7 +3973,7 @@
           <t>CVE-2026-25645</t>
         </is>
       </c>
-      <c r="C47" s="29" t="inlineStr">
+      <c r="C47" s="30" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
@@ -3737,7 +4013,7 @@
           <t>CVE-2026-44431</t>
         </is>
       </c>
-      <c r="C48" s="30" t="inlineStr">
+      <c r="C48" s="31" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
@@ -3793,69 +4069,69 @@
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Report Legend &amp; Attribute Definitions</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="32" t="inlineStr">
+      <c r="A3" s="33" t="inlineStr">
         <is>
           <t>Criticality Levels</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="33" t="inlineStr">
+      <c r="A4" s="34" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="B4" s="34" t="inlineStr">
+      <c r="B4" s="35" t="inlineStr">
         <is>
           <t>Core component; failure causes system-wide outage or critical security breach.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="35" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="B5" s="34" t="inlineStr">
+      <c r="B5" s="35" t="inlineStr">
         <is>
           <t>Important component; failure significantly impacts functionality or security.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="B6" s="34" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>Standard component; moderate impact on operations.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="37" t="inlineStr">
+      <c r="A7" s="38" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="B7" s="34" t="inlineStr">
+      <c r="B7" s="35" t="inlineStr">
         <is>
           <t>Minor or utility component; minimal operational impact.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>21 Client-Required SBOM Attributes</t>
         </is>

</xml_diff>

<commit_message>
fixes the terminal issues
</commit_message>
<xml_diff>
--- a/sbom_output/public/sbom_report.xlsx
+++ b/sbom_output/public/sbom_report.xlsx
@@ -726,7 +726,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CycloneDX v1.5 | Generated: 2026-06-29T08:32:21Z | Report Date: 2026-06-29 14:02</t>
+          <t>CycloneDX v1.5 | Generated: 2026-06-29T09:42:44Z | Report Date: 2026-06-29 15:12</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Author: Client-Assigned Scanning Service  |  Generated: 2026-06-29T08:32:21Z</t>
+          <t>Author: Client-Assigned Scanning Service  |  Generated: 2026-06-29T09:42:44Z</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="S5" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29T08:32:21Z</t>
+          <t>2026-06-29T09:42:44Z</t>
         </is>
       </c>
       <c r="T5" s="20" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="S6" s="23" t="inlineStr">
         <is>
-          <t>2026-06-29T08:32:21Z</t>
+          <t>2026-06-29T09:42:44Z</t>
         </is>
       </c>
       <c r="T6" s="23" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="S7" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29T08:32:21Z</t>
+          <t>2026-06-29T09:42:44Z</t>
         </is>
       </c>
       <c r="T7" s="20" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="S8" s="23" t="inlineStr">
         <is>
-          <t>2026-06-29T08:32:21Z</t>
+          <t>2026-06-29T09:42:44Z</t>
         </is>
       </c>
       <c r="T8" s="23" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="S9" s="20" t="inlineStr">
         <is>
-          <t>2026-06-29T08:32:21Z</t>
+          <t>2026-06-29T09:42:44Z</t>
         </is>
       </c>
       <c r="T9" s="20" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="H10" s="23" t="inlineStr">
         <is>
-          <t>jinja2, urllib3, requests, numpy, django</t>
+          <t>jinja2, numpy, urllib3, requests, django</t>
         </is>
       </c>
       <c r="I10" s="23" t="inlineStr">
@@ -2068,12 +2068,12 @@
       </c>
       <c r="K10" s="22" t="inlineStr">
         <is>
-          <t>2026-06-29T08:32:22.033242Z</t>
+          <t>2026-06-29T09:42:47.425391Z</t>
         </is>
       </c>
       <c r="L10" s="22" t="inlineStr">
         <is>
-          <t>2029-06-28T08:32:22Z</t>
+          <t>2029-06-28T09:42:47Z</t>
         </is>
       </c>
       <c r="M10" s="26" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="S10" s="23" t="inlineStr">
         <is>
-          <t>2026-06-29T08:32:21Z</t>
+          <t>2026-06-29T09:42:44Z</t>
         </is>
       </c>
       <c r="T10" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Implement dynamic executable, archive, and structured property detection, and standardize origin field casing
</commit_message>
<xml_diff>
--- a/sbom_output/public/sbom_report.xlsx
+++ b/sbom_output/public/sbom_report.xlsx
@@ -723,7 +723,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CycloneDX v1.5 | Generated: 2026-06-30T09:11:07Z | Report Date: 2026-06-30 14:41</t>
+          <t>CycloneDX v1.5 | Generated: 2026-06-30T09:47:46Z | Report Date: 2026-06-30 15:17</t>
         </is>
       </c>
     </row>
@@ -1061,9 +1061,9 @@
     <col width="35" customWidth="1" min="18" max="18"/>
     <col width="23" customWidth="1" min="19" max="19"/>
     <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="37" customWidth="1" min="21" max="21"/>
+    <col width="29" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="31" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
     <col width="27" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
     <col width="45" customWidth="1" min="26" max="26"/>
@@ -1082,7 +1082,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Author: Client-Assigned Scanning Service  |  Generated: 2026-06-30T09:11:07Z</t>
+          <t>Author: Client-Assigned Scanning Service  |  Generated: 2026-06-30T09:47:46Z</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="G5" s="20" t="inlineStr">
         <is>
-          <t>open-source</t>
+          <t>Open-Source</t>
         </is>
       </c>
       <c r="H5" s="20" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="S5" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30T09:11:07Z</t>
+          <t>2026-06-30T09:47:46Z</t>
         </is>
       </c>
       <c r="T5" s="20" t="inlineStr">
@@ -1335,17 +1335,17 @@
       </c>
       <c r="U5" s="19" t="inlineStr">
         <is>
-          <t>PyPI package (typically a library)</t>
+          <t>pkg:pypi ecosystem package</t>
         </is>
       </c>
       <c r="V5" s="19" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="W5" s="20" t="inlineStr">
         <is>
-          <t>CycloneDX JSON v1.6 (Merged)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="X5" s="19" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="G6" s="23" t="inlineStr">
         <is>
-          <t>open-source</t>
+          <t>Open-Source</t>
         </is>
       </c>
       <c r="H6" s="23" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="S6" s="23" t="inlineStr">
         <is>
-          <t>2026-06-30T09:11:07Z</t>
+          <t>2026-06-30T09:47:46Z</t>
         </is>
       </c>
       <c r="T6" s="23" t="inlineStr">
@@ -1484,17 +1484,17 @@
       </c>
       <c r="U6" s="22" t="inlineStr">
         <is>
-          <t>PyPI package (typically a library)</t>
+          <t>pkg:pypi ecosystem package</t>
         </is>
       </c>
       <c r="V6" s="22" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="W6" s="23" t="inlineStr">
         <is>
-          <t>CycloneDX JSON v1.6 (Merged)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="X6" s="22" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="G7" s="20" t="inlineStr">
         <is>
-          <t>open-source</t>
+          <t>Open-Source</t>
         </is>
       </c>
       <c r="H7" s="20" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="S7" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30T09:11:07Z</t>
+          <t>2026-06-30T09:47:46Z</t>
         </is>
       </c>
       <c r="T7" s="20" t="inlineStr">
@@ -1633,17 +1633,17 @@
       </c>
       <c r="U7" s="19" t="inlineStr">
         <is>
-          <t>PyPI package (typically a library)</t>
+          <t>pkg:pypi ecosystem package</t>
         </is>
       </c>
       <c r="V7" s="19" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="W7" s="20" t="inlineStr">
         <is>
-          <t>CycloneDX JSON v1.6 (Merged)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="X7" s="19" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="G8" s="23" t="inlineStr">
         <is>
-          <t>open-source</t>
+          <t>Open-Source</t>
         </is>
       </c>
       <c r="H8" s="23" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="S8" s="23" t="inlineStr">
         <is>
-          <t>2026-06-30T09:11:07Z</t>
+          <t>2026-06-30T09:47:46Z</t>
         </is>
       </c>
       <c r="T8" s="23" t="inlineStr">
@@ -1782,17 +1782,17 @@
       </c>
       <c r="U8" s="22" t="inlineStr">
         <is>
-          <t>PyPI package (typically a library)</t>
+          <t>pkg:pypi ecosystem package</t>
         </is>
       </c>
       <c r="V8" s="22" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="W8" s="23" t="inlineStr">
         <is>
-          <t>CycloneDX JSON v1.6 (Merged)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="X8" s="22" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="G9" s="20" t="inlineStr">
         <is>
-          <t>open-source</t>
+          <t>Open-Source</t>
         </is>
       </c>
       <c r="H9" s="20" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="S9" s="20" t="inlineStr">
         <is>
-          <t>2026-06-30T09:11:07Z</t>
+          <t>2026-06-30T09:47:46Z</t>
         </is>
       </c>
       <c r="T9" s="20" t="inlineStr">
@@ -1931,17 +1931,17 @@
       </c>
       <c r="U9" s="19" t="inlineStr">
         <is>
-          <t>PyPI package (typically a library)</t>
+          <t>pkg:pypi ecosystem package</t>
         </is>
       </c>
       <c r="V9" s="19" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="W9" s="20" t="inlineStr">
         <is>
-          <t>CycloneDX JSON v1.6 (Merged)</t>
+          <t>true</t>
         </is>
       </c>
       <c r="X9" s="19" t="inlineStr">

</xml_diff>